<commit_message>
Incidentes verificados por el autor, variante 'solo verificados' y depuración de duplicados
- 10 incidentes verificados con código Almirantazgo; confianza derivada del código (D30)
- Evaluación: variante 'solo verificados' y un evento por día en noticias detectadas (D31)
- Web: etiqueta 'verificado' con el código; selector con tres variantes
- Planilla con los códigos precargados; 18 pruebas; decisiones D30-D32; memoria v0.7

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011eMYWh6VDWd8LKxBrkPUCG
</commit_message>
<xml_diff>
--- a/datos/verificacion/planilla_verificacion.xlsx
+++ b/datos/verificacion/planilla_verificacion.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="273">
   <si>
     <t xml:space="preserve">Planilla de verificación de datos · TFM Monitor Ciber-Geopolítico Argentina</t>
   </si>
@@ -245,6 +245,9 @@
     <t xml:space="preserve">Total de filas</t>
   </si>
   <si>
+    <t xml:space="preserve">Con código Almirantazgo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Revisadas (con decisión)</t>
   </si>
   <si>
@@ -254,7 +257,7 @@
     <t xml:space="preserve">Descartado</t>
   </si>
   <si>
-    <t xml:space="preserve">Avance</t>
+    <t xml:space="preserve">Avance (con código)</t>
   </si>
   <si>
     <t xml:space="preserve">Esta pestaña se calcula sola a partir de la columna «Decisión» de cada pestaña.</t>
@@ -371,6 +374,9 @@
     <t xml:space="preserve">Ya detectado por la plataforma en vivo. Fecha tomada de la nota.</t>
   </si>
   <si>
+    <t xml:space="preserve">2 - Media</t>
+  </si>
+  <si>
     <t xml:space="preserve">INC-021</t>
   </si>
   <si>
@@ -386,6 +392,12 @@
     <t xml:space="preserve">El año (2026) se deduce del día de la semana: verificar.</t>
   </si>
   <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado por el autor el 18/10/2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">INC-020</t>
   </si>
   <si>
@@ -398,9 +410,15 @@
     <t xml:space="preserve">ddos</t>
   </si>
   <si>
+    <t xml:space="preserve">alta</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ocurre 19 días después del anuncio de ingreso al Board of Peace (17/01/2026). La atribución proviene de la SIDE.</t>
   </si>
   <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
     <t xml:space="preserve">INC-019</t>
   </si>
   <si>
@@ -416,9 +434,6 @@
     <t xml:space="preserve">Solo reivindicación del grupo.</t>
   </si>
   <si>
-    <t xml:space="preserve">2 - Media</t>
-  </si>
-  <si>
     <t xml:space="preserve">INC-018</t>
   </si>
   <si>
@@ -432,9 +447,6 @@
   </si>
   <si>
     <t xml:space="preserve">Fuerzas Armadas (datos de unos 50.000 efectivos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">alta</t>
   </si>
   <si>
     <t xml:space="preserve">Un proyecto de Diputados lo sitúa el 13/05/2025.</t>
@@ -1783,37 +1795,37 @@
         <v>72</v>
       </c>
       <c r="B5" s="8" t="n">
+        <f aca="false">COUNTIF(Incidentes!S2:S24,"?*")</f>
+        <v>10</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <f aca="false">COUNTIF('Hechos clave'!N2:N17,"?*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="8" t="n">
         <f aca="false">COUNTA(Incidentes!T2:T24)</f>
         <v>0</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C6" s="8" t="n">
         <f aca="false">COUNTA('Hechos clave'!O2:O17)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B7" s="8" t="n">
         <f aca="false">COUNTIF(Incidentes!T2:T24,"Confirmado")</f>
         <v>0</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C7" s="8" t="n">
         <f aca="false">COUNTIF('Hechos clave'!O2:O17,"Confirmado")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B7" s="8" t="n">
-        <f aca="false">COUNTIF(Incidentes!T2:T24,"Reivindicado sin confirmar")</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <f aca="false">COUNTIF('Hechos clave'!O2:O17,"Reivindicado sin confirmar")</f>
         <v>0</v>
       </c>
     </row>
@@ -1822,11 +1834,11 @@
         <v>74</v>
       </c>
       <c r="B8" s="8" t="n">
-        <f aca="false">COUNTIF(Incidentes!T2:T24,"Descartado")</f>
+        <f aca="false">COUNTIF(Incidentes!T2:T24,"Reivindicado sin confirmar")</f>
         <v>0</v>
       </c>
       <c r="C8" s="8" t="n">
-        <f aca="false">COUNTIF('Hechos clave'!O2:O17,"Descartado")</f>
+        <f aca="false">COUNTIF('Hechos clave'!O2:O17,"Reivindicado sin confirmar")</f>
         <v>0</v>
       </c>
     </row>
@@ -1834,18 +1846,31 @@
       <c r="A9" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
+        <f aca="false">COUNTIF(Incidentes!T2:T24,"Descartado")</f>
+        <v>0</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <f aca="false">COUNTIF('Hechos clave'!O2:O17,"Descartado")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="9" t="n">
         <f aca="false">IF(B4=0,0,B5/B4)</f>
-        <v>0</v>
-      </c>
-      <c r="C9" s="9" t="n">
+        <v>0.434782608695652</v>
+      </c>
+      <c r="C10" s="9" t="n">
         <f aca="false">IF(C4=0,0,C5/C4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1887,43 +1912,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L1" s="12" t="s">
         <v>50</v>
       </c>
       <c r="M1" s="12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="N1" s="12" t="s">
         <v>54</v>
@@ -1932,13 +1957,13 @@
         <v>55</v>
       </c>
       <c r="P1" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q1" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="R1" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="S1" s="12" t="s">
         <v>62</v>
@@ -1952,37 +1977,37 @@
     </row>
     <row r="2" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I2" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J2" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K2" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L2" s="15"/>
       <c r="M2" s="15"/>
@@ -2000,37 +2025,37 @@
     </row>
     <row r="3" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I3" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K3" s="13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L3" s="15"/>
       <c r="M3" s="15"/>
@@ -2048,421 +2073,469 @@
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="L4" s="15"/>
       <c r="M4" s="15"/>
       <c r="N4" s="15"/>
       <c r="O4" s="15"/>
       <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
-      <c r="R4" s="15"/>
+      <c r="Q4" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="R4" s="15" t="n">
+        <v>3</v>
+      </c>
       <c r="S4" s="16" t="str">
         <f aca="false">IF(OR(Q4="",R4=""),"",Q4&amp;R4)</f>
-        <v/>
+        <v>C3</v>
       </c>
       <c r="T4" s="15"/>
-      <c r="U4" s="15"/>
+      <c r="U4" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>53</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="I5" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="L5" s="15"/>
       <c r="M5" s="15"/>
       <c r="N5" s="15"/>
       <c r="O5" s="15"/>
       <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
+      <c r="Q5" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="R5" s="15" t="n">
+        <v>2</v>
+      </c>
       <c r="S5" s="16" t="str">
         <f aca="false">IF(OR(Q5="",R5=""),"",Q5&amp;R5)</f>
-        <v/>
+        <v>B2</v>
       </c>
       <c r="T5" s="15"/>
-      <c r="U5" s="15"/>
+      <c r="U5" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="L6" s="15"/>
       <c r="M6" s="15"/>
       <c r="N6" s="15"/>
       <c r="O6" s="15"/>
       <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="15"/>
+      <c r="Q6" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="R6" s="15" t="n">
+        <v>4</v>
+      </c>
       <c r="S6" s="16" t="str">
         <f aca="false">IF(OR(Q6="",R6=""),"",Q6&amp;R6)</f>
-        <v/>
+        <v>C4</v>
       </c>
       <c r="T6" s="15"/>
-      <c r="U6" s="15"/>
+      <c r="U6" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="L7" s="15"/>
       <c r="M7" s="15"/>
       <c r="N7" s="15"/>
       <c r="O7" s="15"/>
       <c r="P7" s="15"/>
-      <c r="Q7" s="15"/>
-      <c r="R7" s="15"/>
+      <c r="Q7" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="R7" s="15" t="n">
+        <v>2</v>
+      </c>
       <c r="S7" s="16" t="str">
         <f aca="false">IF(OR(Q7="",R7=""),"",Q7&amp;R7)</f>
-        <v/>
+        <v>B2</v>
       </c>
       <c r="T7" s="15"/>
-      <c r="U7" s="15"/>
+      <c r="U7" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C8" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="F8" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="D8" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>132</v>
-      </c>
       <c r="G8" s="13" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
       <c r="N8" s="15"/>
       <c r="O8" s="15"/>
       <c r="P8" s="15"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="15"/>
+      <c r="Q8" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="R8" s="15" t="n">
+        <v>1</v>
+      </c>
       <c r="S8" s="16" t="str">
         <f aca="false">IF(OR(Q8="",R8=""),"",Q8&amp;R8)</f>
-        <v/>
+        <v>A1</v>
       </c>
       <c r="T8" s="15"/>
-      <c r="U8" s="15"/>
+      <c r="U8" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="L9" s="15"/>
       <c r="M9" s="15"/>
       <c r="N9" s="15"/>
       <c r="O9" s="15"/>
       <c r="P9" s="15"/>
-      <c r="Q9" s="15"/>
-      <c r="R9" s="15"/>
+      <c r="Q9" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="R9" s="15" t="n">
+        <v>4</v>
+      </c>
       <c r="S9" s="16" t="str">
         <f aca="false">IF(OR(Q9="",R9=""),"",Q9&amp;R9)</f>
-        <v/>
+        <v>B4</v>
       </c>
       <c r="T9" s="15"/>
-      <c r="U9" s="15"/>
+      <c r="U9" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
       <c r="N10" s="15"/>
       <c r="O10" s="15"/>
       <c r="P10" s="15"/>
-      <c r="Q10" s="15"/>
-      <c r="R10" s="15"/>
+      <c r="Q10" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="R10" s="15" t="n">
+        <v>1</v>
+      </c>
       <c r="S10" s="16" t="str">
         <f aca="false">IF(OR(Q10="",R10=""),"",Q10&amp;R10)</f>
-        <v/>
+        <v>A1</v>
       </c>
       <c r="T10" s="15"/>
-      <c r="U10" s="15"/>
+      <c r="U10" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
       <c r="N11" s="15"/>
       <c r="O11" s="15"/>
       <c r="P11" s="15"/>
-      <c r="Q11" s="15"/>
-      <c r="R11" s="15"/>
+      <c r="Q11" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="R11" s="15" t="n">
+        <v>3</v>
+      </c>
       <c r="S11" s="16" t="str">
         <f aca="false">IF(OR(Q11="",R11=""),"",Q11&amp;R11)</f>
-        <v/>
+        <v>B3</v>
       </c>
       <c r="T11" s="15"/>
-      <c r="U11" s="15"/>
+      <c r="U11" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K12" s="13" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
@@ -2480,37 +2553,37 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C13" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D13" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>158</v>
-      </c>
       <c r="F13" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
@@ -2528,37 +2601,37 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
@@ -2576,37 +2649,37 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
@@ -2624,37 +2697,37 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
@@ -2672,37 +2745,37 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
@@ -2720,37 +2793,37 @@
     </row>
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
@@ -2768,37 +2841,37 @@
     </row>
     <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J19" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
@@ -2816,133 +2889,145 @@
     </row>
     <row r="20" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J20" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
       <c r="N20" s="15"/>
       <c r="O20" s="15"/>
       <c r="P20" s="15"/>
-      <c r="Q20" s="15"/>
-      <c r="R20" s="15"/>
+      <c r="Q20" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="R20" s="15" t="n">
+        <v>1</v>
+      </c>
       <c r="S20" s="16" t="str">
         <f aca="false">IF(OR(Q20="",R20=""),"",Q20&amp;R20)</f>
-        <v/>
+        <v>A1</v>
       </c>
       <c r="T20" s="15"/>
-      <c r="U20" s="15"/>
+      <c r="U20" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
       <c r="N21" s="15"/>
       <c r="O21" s="15"/>
       <c r="P21" s="15"/>
-      <c r="Q21" s="15"/>
-      <c r="R21" s="15"/>
+      <c r="Q21" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="R21" s="15" t="n">
+        <v>1</v>
+      </c>
       <c r="S21" s="16" t="str">
         <f aca="false">IF(OR(Q21="",R21=""),"",Q21&amp;R21)</f>
-        <v/>
+        <v>A1</v>
       </c>
       <c r="T21" s="15"/>
-      <c r="U21" s="15"/>
+      <c r="U21" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J22" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K22" s="13" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
@@ -2960,37 +3045,37 @@
     </row>
     <row r="23" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
@@ -3008,37 +3093,37 @@
     </row>
     <row r="24" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B24" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="C24" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="C24" s="13" t="s">
-        <v>206</v>
-      </c>
       <c r="D24" s="13" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J24" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K24" s="13" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
@@ -3149,28 +3234,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>50</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I1" s="12" t="s">
         <v>54</v>
@@ -3179,13 +3264,13 @@
         <v>55</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="L1" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="M1" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N1" s="12" t="s">
         <v>62</v>
@@ -3199,22 +3284,22 @@
     </row>
     <row r="2" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
@@ -3232,22 +3317,22 @@
     </row>
     <row r="3" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D3" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="E3" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="E3" s="13" t="s">
-        <v>220</v>
-      </c>
       <c r="F3" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
@@ -3265,22 +3350,22 @@
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="D4" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="E4" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="E4" s="13" t="s">
-        <v>220</v>
-      </c>
       <c r="F4" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G4" s="15"/>
       <c r="H4" s="15"/>
@@ -3298,22 +3383,22 @@
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="D5" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="D5" s="13" t="s">
+      <c r="E5" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="E5" s="13" t="s">
-        <v>220</v>
-      </c>
       <c r="F5" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
@@ -3331,22 +3416,22 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
@@ -3364,22 +3449,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G7" s="15"/>
       <c r="H7" s="15"/>
@@ -3397,22 +3482,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D8" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="E8" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="E8" s="13" t="s">
-        <v>220</v>
-      </c>
       <c r="F8" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
@@ -3430,22 +3515,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G9" s="15"/>
       <c r="H9" s="15"/>
@@ -3463,22 +3548,22 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G10" s="15"/>
       <c r="H10" s="15"/>
@@ -3496,22 +3581,22 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G11" s="15"/>
       <c r="H11" s="15"/>
@@ -3529,22 +3614,22 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G12" s="15"/>
       <c r="H12" s="15"/>
@@ -3562,22 +3647,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G13" s="15"/>
       <c r="H13" s="15"/>
@@ -3595,22 +3680,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G14" s="15"/>
       <c r="H14" s="15"/>
@@ -3628,22 +3713,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G15" s="15"/>
       <c r="H15" s="15"/>
@@ -3661,22 +3746,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="15"/>
@@ -3694,22 +3779,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G17" s="15"/>
       <c r="H17" s="15"/>

</xml_diff>

<commit_message>
Verificación de incidentes hacktivistas: 4 verificados y 2 descartados
- INC-002, INC-004, INC-005: D3; INC-006: D2
- INC-001 e INC-003 descartados (no relacionados con el Estado argentino): se listan con
  su motivo pero no entran al cálculo (D33)
- Planilla y memoria v0.8 actualizadas; 19 pruebas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011eMYWh6VDWd8LKxBrkPUCG
</commit_message>
<xml_diff>
--- a/datos/verificacion/planilla_verificacion.xlsx
+++ b/datos/verificacion/planilla_verificacion.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="275">
   <si>
     <t xml:space="preserve">Planilla de verificación de datos · TFM Monitor Ciber-Geopolítico Argentina</t>
   </si>
@@ -527,6 +527,9 @@
     <t xml:space="preserve">Posterior al período de estudio.</t>
   </si>
   <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
     <t xml:space="preserve">INC-004</t>
   </si>
   <si>
@@ -657,6 +660,9 @@
   </si>
   <si>
     <t xml:space="preserve">Falta el día exacto y una segunda fuente. Verificar el dominio afectado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No guarda relación con el Estado argentino (verificación del autor, 18/10/2026).</t>
   </si>
   <si>
     <t xml:space="preserve">INC-003</t>
@@ -1118,7 +1124,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1178,6 +1184,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1796,7 +1810,7 @@
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">COUNTIF(Incidentes!S2:S24,"?*")</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">COUNTIF('Hechos clave'!N2:N17,"?*")</f>
@@ -1809,7 +1823,7 @@
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">COUNTA(Incidentes!T2:T24)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">COUNTA('Hechos clave'!O2:O17)</f>
@@ -1848,7 +1862,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">COUNTIF(Incidentes!T2:T24,"Descartado")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C9" s="8" t="n">
         <f aca="false">COUNTIF('Hechos clave'!O2:O17,"Descartado")</f>
@@ -1861,7 +1875,7 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">IF(B4=0,0,B5/B4)</f>
-        <v>0.434782608695652</v>
+        <v>0.608695652173913</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">IF(C4=0,0,C5/C4)</f>
@@ -2532,7 +2546,7 @@
         <v>101</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="K12" s="13" t="s">
         <v>164</v>
@@ -2542,24 +2556,30 @@
       <c r="N12" s="15"/>
       <c r="O12" s="15"/>
       <c r="P12" s="15"/>
-      <c r="Q12" s="15"/>
-      <c r="R12" s="15"/>
+      <c r="Q12" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="R12" s="15" t="n">
+        <v>3</v>
+      </c>
       <c r="S12" s="16" t="str">
         <f aca="false">IF(OR(Q12="",R12=""),"",Q12&amp;R12)</f>
-        <v/>
+        <v>D3</v>
       </c>
       <c r="T12" s="15"/>
-      <c r="U12" s="15"/>
+      <c r="U12" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
         <v>104</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>96</v>
@@ -2571,10 +2591,10 @@
         <v>109</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I13" s="14" t="s">
         <v>101</v>
@@ -2583,34 +2603,40 @@
         <v>102</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
       <c r="N13" s="15"/>
       <c r="O13" s="15"/>
       <c r="P13" s="15"/>
-      <c r="Q13" s="15"/>
-      <c r="R13" s="15"/>
+      <c r="Q13" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="R13" s="15" t="n">
+        <v>3</v>
+      </c>
       <c r="S13" s="16" t="str">
         <f aca="false">IF(OR(Q13="",R13=""),"",Q13&amp;R13)</f>
-        <v/>
+        <v>D3</v>
       </c>
       <c r="T13" s="15"/>
-      <c r="U13" s="15"/>
+      <c r="U13" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
         <v>104</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E14" s="13" t="s">
         <v>162</v>
@@ -2619,7 +2645,7 @@
         <v>109</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H14" s="13" t="s">
         <v>144</v>
@@ -2631,31 +2657,37 @@
         <v>102</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
       <c r="N14" s="15"/>
       <c r="O14" s="15"/>
       <c r="P14" s="15"/>
-      <c r="Q14" s="15"/>
-      <c r="R14" s="15"/>
+      <c r="Q14" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="R14" s="15" t="n">
+        <v>2</v>
+      </c>
       <c r="S14" s="16" t="str">
         <f aca="false">IF(OR(Q14="",R14=""),"",Q14&amp;R14)</f>
-        <v/>
+        <v>D2</v>
       </c>
       <c r="T14" s="15"/>
-      <c r="U14" s="15"/>
+      <c r="U14" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
         <v>93</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>96</v>
@@ -2667,7 +2699,7 @@
         <v>137</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H15" s="13" t="s">
         <v>100</v>
@@ -2679,7 +2711,7 @@
         <v>102</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
@@ -2700,10 +2732,10 @@
         <v>114</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>107</v>
@@ -2715,7 +2747,7 @@
         <v>98</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H16" s="13" t="s">
         <v>111</v>
@@ -2727,7 +2759,7 @@
         <v>126</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
@@ -2748,10 +2780,10 @@
         <v>114</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>107</v>
@@ -2763,7 +2795,7 @@
         <v>98</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H17" s="13" t="s">
         <v>111</v>
@@ -2775,7 +2807,7 @@
         <v>112</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
@@ -2796,10 +2828,10 @@
         <v>104</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>107</v>
@@ -2811,7 +2843,7 @@
         <v>109</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>111</v>
@@ -2820,34 +2852,40 @@
         <v>101</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
       <c r="N18" s="15"/>
       <c r="O18" s="15"/>
       <c r="P18" s="15"/>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="15"/>
+      <c r="Q18" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="R18" s="15" t="n">
+        <v>3</v>
+      </c>
       <c r="S18" s="16" t="str">
         <f aca="false">IF(OR(Q18="",R18=""),"",Q18&amp;R18)</f>
-        <v/>
+        <v>D3</v>
       </c>
       <c r="T18" s="15"/>
-      <c r="U18" s="15"/>
+      <c r="U18" s="15" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
         <v>114</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>96</v>
@@ -2859,7 +2897,7 @@
         <v>137</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>111</v>
@@ -2871,7 +2909,7 @@
         <v>126</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
@@ -2892,10 +2930,10 @@
         <v>114</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>96</v>
@@ -2907,7 +2945,7 @@
         <v>137</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H20" s="13" t="s">
         <v>144</v>
@@ -2919,7 +2957,7 @@
         <v>126</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
@@ -2946,22 +2984,22 @@
         <v>114</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D21" s="13" t="s">
         <v>96</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>98</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H21" s="13" t="s">
         <v>100</v>
@@ -2973,7 +3011,7 @@
         <v>126</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
@@ -3000,22 +3038,22 @@
         <v>104</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F22" s="13" t="s">
         <v>109</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>144</v>
@@ -3027,7 +3065,7 @@
         <v>102</v>
       </c>
       <c r="K22" s="13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
@@ -3040,30 +3078,34 @@
         <f aca="false">IF(OR(Q22="",R22=""),"",Q22&amp;R22)</f>
         <v/>
       </c>
-      <c r="T22" s="15"/>
-      <c r="U22" s="15"/>
+      <c r="T22" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="U22" s="15" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
         <v>104</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F23" s="13" t="s">
         <v>109</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H23" s="13" t="s">
         <v>111</v>
@@ -3075,7 +3117,7 @@
         <v>102</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
@@ -3088,30 +3130,34 @@
         <f aca="false">IF(OR(Q23="",R23=""),"",Q23&amp;R23)</f>
         <v/>
       </c>
-      <c r="T23" s="15"/>
-      <c r="U23" s="15"/>
+      <c r="T23" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="U23" s="15" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
         <v>104</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F24" s="13" t="s">
         <v>109</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="H24" s="13" t="s">
         <v>125</v>
@@ -3123,7 +3169,7 @@
         <v>102</v>
       </c>
       <c r="K24" s="13" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15"/>
@@ -3142,10 +3188,10 @@
   </sheetData>
   <autoFilter ref="A1:U24"/>
   <conditionalFormatting sqref="T2:T24">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>T2="Confirmado"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>T2="Descartado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3240,10 +3286,10 @@
         <v>80</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>86</v>
@@ -3284,19 +3330,19 @@
     </row>
     <row r="2" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F2" s="13" t="s">
         <v>126</v>
@@ -3317,19 +3363,19 @@
     </row>
     <row r="3" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B3" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="E3" s="13" t="s">
         <v>226</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>227</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>224</v>
       </c>
       <c r="F3" s="13" t="s">
         <v>112</v>
@@ -3350,19 +3396,19 @@
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B4" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>231</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>228</v>
-      </c>
       <c r="E4" s="13" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F4" s="13" t="s">
         <v>112</v>
@@ -3383,19 +3429,19 @@
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F5" s="13" t="s">
         <v>126</v>
@@ -3416,19 +3462,19 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F6" s="13" t="s">
         <v>126</v>
@@ -3449,19 +3495,19 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F7" s="13" t="s">
         <v>126</v>
@@ -3482,19 +3528,19 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>112</v>
@@ -3515,19 +3561,19 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F9" s="13" t="s">
         <v>126</v>
@@ -3548,16 +3594,16 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E10" s="14" t="s">
         <v>101</v>
@@ -3581,16 +3627,16 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E11" s="14" t="s">
         <v>101</v>
@@ -3614,16 +3660,16 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E12" s="14" t="s">
         <v>101</v>
@@ -3647,16 +3693,16 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>101</v>
@@ -3680,16 +3726,16 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>101</v>
@@ -3713,16 +3759,16 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E15" s="14" t="s">
         <v>101</v>
@@ -3746,16 +3792,16 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>101</v>
@@ -3779,16 +3825,16 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>101</v>
@@ -3813,10 +3859,10 @@
   </sheetData>
   <autoFilter ref="A1:P17"/>
   <conditionalFormatting sqref="O2:O17">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>O2="Confirmado"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>O2="Descartado"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
INC-022 verificado (B1) y descartado: la AFA no es un organismo del Estado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011eMYWh6VDWd8LKxBrkPUCG
</commit_message>
<xml_diff>
--- a/datos/verificacion/planilla_verificacion.xlsx
+++ b/datos/verificacion/planilla_verificacion.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="275">
   <si>
     <t xml:space="preserve">Planilla de verificación de datos · TFM Monitor Ciber-Geopolítico Argentina</t>
   </si>
@@ -368,36 +368,42 @@
     <t xml:space="preserve">filtracion</t>
   </si>
   <si>
+    <t xml:space="preserve">alta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ya detectado por la plataforma en vivo. Fecha tomada de la nota.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificado por el autor el 18/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 - Media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INC-021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Gentlemen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IBR-CONICET (Rosario)</t>
+  </si>
+  <si>
     <t xml:space="preserve">media</t>
   </si>
   <si>
-    <t xml:space="preserve">Ya detectado por la plataforma en vivo. Fecha tomada de la nota.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 - Media</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INC-021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Gentlemen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IBR-CONICET (Rosario)</t>
-  </si>
-  <si>
     <t xml:space="preserve">El año (2026) se deduce del día de la semana: verificar.</t>
   </si>
   <si>
     <t xml:space="preserve">C</t>
   </si>
   <si>
-    <t xml:space="preserve">Verificado por el autor el 18/10/2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">INC-020</t>
   </si>
   <si>
@@ -410,13 +416,7 @@
     <t xml:space="preserve">ddos</t>
   </si>
   <si>
-    <t xml:space="preserve">alta</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ocurre 19 días después del anuncio de ingreso al Board of Peace (17/01/2026). La atribución proviene de la SIDE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B</t>
   </si>
   <si>
     <t xml:space="preserve">INC-019</t>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">COUNTIF(Incidentes!S2:S24,"?*")</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">COUNTIF('Hechos clave'!N2:N17,"?*")</f>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">COUNTA(Incidentes!T2:T24)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">COUNTA('Hechos clave'!O2:O17)</f>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">COUNTIF(Incidentes!T2:T24,"Descartado")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" s="8" t="n">
         <f aca="false">COUNTIF('Hechos clave'!O2:O17,"Descartado")</f>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">IF(B4=0,0,B5/B4)</f>
-        <v>0.608695652173913</v>
+        <v>0.652173913043478</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">IF(C4=0,0,C5/C4)</f>
@@ -2076,36 +2076,44 @@
       <c r="N3" s="15"/>
       <c r="O3" s="15"/>
       <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="15"/>
+      <c r="Q3" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="R3" s="15" t="n">
+        <v>1</v>
+      </c>
       <c r="S3" s="16" t="str">
         <f aca="false">IF(OR(Q3="",R3=""),"",Q3&amp;R3)</f>
-        <v/>
-      </c>
-      <c r="T3" s="15"/>
-      <c r="U3" s="15"/>
+        <v>B1</v>
+      </c>
+      <c r="T3" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="U3" s="15" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>107</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F4" s="13" t="s">
         <v>98</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H4" s="13" t="s">
         <v>100</v>
@@ -2114,10 +2122,10 @@
         <v>101</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="L4" s="15"/>
       <c r="M4" s="15"/>
@@ -2125,7 +2133,7 @@
       <c r="O4" s="15"/>
       <c r="P4" s="15"/>
       <c r="Q4" s="15" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="R4" s="15" t="n">
         <v>3</v>
@@ -2136,7 +2144,7 @@
       </c>
       <c r="T4" s="15"/>
       <c r="U4" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2144,7 +2152,7 @@
         <v>104</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>53</v>
@@ -2153,25 +2161,25 @@
         <v>96</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F5" s="13" t="s">
         <v>109</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I5" s="14" t="s">
         <v>101</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L5" s="15"/>
       <c r="M5" s="15"/>
@@ -2179,7 +2187,7 @@
       <c r="O5" s="15"/>
       <c r="P5" s="15"/>
       <c r="Q5" s="15" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="R5" s="15" t="n">
         <v>2</v>
@@ -2190,7 +2198,7 @@
       </c>
       <c r="T5" s="15"/>
       <c r="U5" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2233,7 +2241,7 @@
       <c r="O6" s="15"/>
       <c r="P6" s="15"/>
       <c r="Q6" s="15" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="R6" s="15" t="n">
         <v>4</v>
@@ -2244,12 +2252,12 @@
       </c>
       <c r="T6" s="15"/>
       <c r="U6" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>134</v>
@@ -2276,7 +2284,7 @@
         <v>101</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="K7" s="13" t="s">
         <v>139</v>
@@ -2287,7 +2295,7 @@
       <c r="O7" s="15"/>
       <c r="P7" s="15"/>
       <c r="Q7" s="15" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="R7" s="15" t="n">
         <v>2</v>
@@ -2298,12 +2306,12 @@
       </c>
       <c r="T7" s="15"/>
       <c r="U7" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>140</v>
@@ -2330,7 +2338,7 @@
         <v>101</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="K8" s="13" t="s">
         <v>145</v>
@@ -2352,7 +2360,7 @@
       </c>
       <c r="T8" s="15"/>
       <c r="U8" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2395,7 +2403,7 @@
       <c r="O9" s="15"/>
       <c r="P9" s="15"/>
       <c r="Q9" s="15" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="R9" s="15" t="n">
         <v>4</v>
@@ -2406,12 +2414,12 @@
       </c>
       <c r="T9" s="15"/>
       <c r="U9" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>150</v>
@@ -2438,7 +2446,7 @@
         <v>101</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="K10" s="13" t="s">
         <v>154</v>
@@ -2460,12 +2468,12 @@
       </c>
       <c r="T10" s="15"/>
       <c r="U10" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>155</v>
@@ -2492,7 +2500,7 @@
         <v>101</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="K11" s="13" t="s">
         <v>159</v>
@@ -2503,7 +2511,7 @@
       <c r="O11" s="15"/>
       <c r="P11" s="15"/>
       <c r="Q11" s="15" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="R11" s="15" t="n">
         <v>3</v>
@@ -2514,7 +2522,7 @@
       </c>
       <c r="T11" s="15"/>
       <c r="U11" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2568,7 +2576,7 @@
       </c>
       <c r="T12" s="15"/>
       <c r="U12" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2622,7 +2630,7 @@
       </c>
       <c r="T13" s="15"/>
       <c r="U13" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2676,7 +2684,7 @@
       </c>
       <c r="T14" s="15"/>
       <c r="U14" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2729,7 +2737,7 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>180</v>
@@ -2756,7 +2764,7 @@
         <v>101</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="K16" s="13" t="s">
         <v>183</v>
@@ -2777,7 +2785,7 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B17" s="13" t="s">
         <v>184</v>
@@ -2804,7 +2812,7 @@
         <v>101</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="K17" s="13" t="s">
         <v>187</v>
@@ -2874,12 +2882,12 @@
       </c>
       <c r="T18" s="15"/>
       <c r="U18" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>192</v>
@@ -2906,7 +2914,7 @@
         <v>101</v>
       </c>
       <c r="J19" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="K19" s="13" t="s">
         <v>195</v>
@@ -2927,7 +2935,7 @@
     </row>
     <row r="20" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>196</v>
@@ -2954,7 +2962,7 @@
         <v>101</v>
       </c>
       <c r="J20" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="K20" s="13" t="s">
         <v>199</v>
@@ -2976,12 +2984,12 @@
       </c>
       <c r="T20" s="15"/>
       <c r="U20" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B21" s="13" t="s">
         <v>200</v>
@@ -3008,7 +3016,7 @@
         <v>101</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="K21" s="13" t="s">
         <v>204</v>
@@ -3030,7 +3038,7 @@
       </c>
       <c r="T21" s="15"/>
       <c r="U21" s="15" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3160,7 +3168,7 @@
         <v>218</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I24" s="14" t="s">
         <v>101</v>
@@ -3345,7 +3353,7 @@
         <v>226</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G2" s="15"/>
       <c r="H2" s="15"/>
@@ -3378,7 +3386,7 @@
         <v>226</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
@@ -3411,7 +3419,7 @@
         <v>226</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="G4" s="15"/>
       <c r="H4" s="15"/>
@@ -3444,7 +3452,7 @@
         <v>226</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
@@ -3477,7 +3485,7 @@
         <v>226</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
@@ -3510,7 +3518,7 @@
         <v>226</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G7" s="15"/>
       <c r="H7" s="15"/>
@@ -3543,7 +3551,7 @@
         <v>226</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
@@ -3576,7 +3584,7 @@
         <v>226</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G9" s="15"/>
       <c r="H9" s="15"/>
@@ -3609,7 +3617,7 @@
         <v>101</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G10" s="15"/>
       <c r="H10" s="15"/>
@@ -3642,7 +3650,7 @@
         <v>101</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="G11" s="15"/>
       <c r="H11" s="15"/>
@@ -3675,7 +3683,7 @@
         <v>101</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G12" s="15"/>
       <c r="H12" s="15"/>
@@ -3708,7 +3716,7 @@
         <v>101</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="G13" s="15"/>
       <c r="H13" s="15"/>
@@ -3741,7 +3749,7 @@
         <v>101</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G14" s="15"/>
       <c r="H14" s="15"/>
@@ -3774,7 +3782,7 @@
         <v>101</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="G15" s="15"/>
       <c r="H15" s="15"/>
@@ -3807,7 +3815,7 @@
         <v>101</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="15"/>
@@ -3840,7 +3848,7 @@
         <v>101</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G17" s="15"/>
       <c r="H17" s="15"/>

</xml_diff>